<commit_message>
reorganized and renamed things
</commit_message>
<xml_diff>
--- a/data/example/data.xlsx
+++ b/data/example/data.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/march/workspace/git/TT/GroupFormation/data/example/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4814BCC0-85D6-8B43-BB7D-A02BF0F50BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2B0B27-A58E-A54F-B865-2E6D08782D62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="26080" windowHeight="18400" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="26080" windowHeight="18400" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="students" sheetId="1" r:id="rId1"/>
     <sheet name="dtypes" sheetId="2" r:id="rId2"/>
-    <sheet name="projects" sheetId="3" r:id="rId3"/>
+    <sheet name="teams" sheetId="3" r:id="rId3"/>
     <sheet name="types" sheetId="4" r:id="rId4"/>
     <sheet name="restrictions" sheetId="5" r:id="rId5"/>
   </sheets>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="48">
   <si>
     <t>grp_id</t>
   </si>
@@ -139,12 +139,6 @@
     <t>float64</t>
   </si>
   <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>team</t>
-  </si>
-  <si>
     <t>title</t>
   </si>
   <si>
@@ -154,21 +148,6 @@
     <t>max_cap</t>
   </si>
   <si>
-    <t>prj_id</t>
-  </si>
-  <si>
-    <t>instit</t>
-  </si>
-  <si>
-    <t>institute</t>
-  </si>
-  <si>
-    <t>mini</t>
-  </si>
-  <si>
-    <t>wl</t>
-  </si>
-  <si>
     <t>p1</t>
   </si>
   <si>
@@ -181,7 +160,19 @@
     <t>2a</t>
   </si>
   <si>
-    <t>key</t>
+    <t>team_type</t>
+  </si>
+  <si>
+    <t>student_type</t>
+  </si>
+  <si>
+    <t>team_id</t>
+  </si>
+  <si>
+    <t>team_group</t>
+  </si>
+  <si>
+    <t>team_subgroup</t>
   </si>
 </sst>
 </file>
@@ -904,45 +895,33 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" t="s">
         <v>36</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>37</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>38</v>
-      </c>
-      <c r="D1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E1" t="s">
-        <v>40</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
       </c>
       <c r="G1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H1" t="s">
-        <v>42</v>
-      </c>
-      <c r="I1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J1" t="s">
-        <v>44</v>
-      </c>
-      <c r="K1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -950,7 +929,7 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D2">
         <v>2</v>
@@ -962,10 +941,10 @@
         <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -973,7 +952,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -985,7 +964,7 @@
         <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1001,10 +980,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B1" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>